<commit_message>
Guide 1.1 from pilot findings; pilot rechecked
</commit_message>
<xml_diff>
--- a/data/labels/arrangement_dev_pilot.xlsx
+++ b/data/labels/arrangement_dev_pilot.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="74">
   <si>
     <t>sample_id</t>
   </si>
@@ -40,15 +40,21 @@
     <t>no</t>
   </si>
   <si>
+    <t>unclear</t>
+  </si>
+  <si>
+    <t>On-site SEO can mean SEO work on the website, so physical attendance is unclear.</t>
+  </si>
+  <si>
+    <t>A002</t>
+  </si>
+  <si>
+    <t>Virtual Assistant Wanted: Make an Impact from Anywhere</t>
+  </si>
+  <si>
     <t>yes</t>
   </si>
   <si>
-    <t>A002</t>
-  </si>
-  <si>
-    <t>Virtual Assistant Wanted: Make an Impact from Anywhere</t>
-  </si>
-  <si>
     <t>A003</t>
   </si>
   <si>
@@ -151,6 +157,9 @@
     <t>Remote Team Manager &amp; GIS Analyst with Python Skills</t>
   </si>
   <si>
+    <t>Remote describes the team being managed, not clearly the worker’s location.</t>
+  </si>
+  <si>
     <t>A020</t>
   </si>
   <si>
@@ -181,6 +190,9 @@
     <t>IT &amp; Remote Networking Expert</t>
   </si>
   <si>
+    <t>Remote networking is a technical term, not a work-arrangement requirement.</t>
+  </si>
+  <si>
     <t>A025</t>
   </si>
   <si>
@@ -206,6 +218,9 @@
   </si>
   <si>
     <t>Onsite Wordpress SEO Specialist</t>
+  </si>
+  <si>
+    <t>Onsite SEO can mean SEO work on the website, so physical attendance is unclear.</t>
   </si>
   <si>
     <t>A029</t>
@@ -548,16 +563,19 @@
       <c r="E2" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="F2" s="4" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>8</v>
@@ -568,10 +586,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>8</v>
@@ -585,10 +603,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>8</v>
@@ -602,10 +620,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>8</v>
@@ -619,10 +637,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>8</v>
@@ -636,13 +654,13 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>8</v>
@@ -653,13 +671,13 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>8</v>
@@ -670,16 +688,16 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>8</v>
@@ -687,10 +705,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>8</v>
@@ -704,13 +722,13 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>8</v>
@@ -721,10 +739,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>8</v>
@@ -738,13 +756,13 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>8</v>
@@ -755,10 +773,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>8</v>
@@ -772,10 +790,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>8</v>
@@ -784,18 +802,18 @@
         <v>8</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>8</v>
@@ -806,10 +824,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>8</v>
@@ -823,10 +841,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>8</v>
@@ -835,32 +853,35 @@
         <v>8</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>8</v>
@@ -869,18 +890,18 @@
         <v>8</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>8</v>
@@ -891,16 +912,16 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>8</v>
@@ -908,13 +929,13 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>8</v>
@@ -925,27 +946,30 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>8</v>
@@ -957,18 +981,18 @@
         <v>8</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>8</v>
@@ -979,10 +1003,10 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>8</v>
@@ -996,10 +1020,10 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>8</v>
@@ -1010,16 +1034,19 @@
       <c r="E29" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="F29" s="4" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>8</v>
@@ -1030,16 +1057,16 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>8</v>

</xml_diff>